<commit_message>
Worked on the company wise feature
</commit_message>
<xml_diff>
--- a/src/modules/questions/templates/question_template.xlsx
+++ b/src/modules/questions/templates/question_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="62">
   <si>
     <t>subject</t>
   </si>
@@ -32,12 +32,15 @@
     <t>correctAnswer</t>
   </si>
   <si>
-    <t>marks</t>
-  </si>
-  <si>
     <t>difficulty</t>
   </si>
   <si>
+    <t>company</t>
+  </si>
+  <si>
+    <t>imageUrl</t>
+  </si>
+  <si>
     <t>Mathematics</t>
   </si>
   <si>
@@ -56,12 +59,12 @@
     <t>4</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>EASY</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>Science</t>
   </si>
   <si>
@@ -119,12 +122,18 @@
     <t>Geometry</t>
   </si>
   <si>
-    <t>Number of sides in a square</t>
+    <t>Number of sides in a square (see image)</t>
   </si>
   <si>
     <t>2|3|4|5</t>
   </si>
   <si>
+    <t>TCS</t>
+  </si>
+  <si>
+    <t>https://example.com/images/square.png</t>
+  </si>
+  <si>
     <t>Biology</t>
   </si>
   <si>
@@ -155,16 +164,19 @@
     <t>The correct answer value (e.g., "4" for MCQ, "TRUE" for TRUE_FALSE)</t>
   </si>
   <si>
-    <t>Positive number</t>
-  </si>
-  <si>
     <t>EASY, MEDIUM, or HARD</t>
   </si>
   <si>
+    <t>Optional. The name of an existing company to tag this question with (e.g., TCS, Infosys). Must match an existing company name. Leave blank if not applicable.</t>
+  </si>
+  <si>
+    <t>Optional. A direct link to an image (e.g., a diagram) to show below the question text. Leave blank if not needed.</t>
+  </si>
+  <si>
     <t>Important Notes:</t>
   </si>
   <si>
-    <t>- All fields are required</t>
+    <t>- All fields are required except company and imageUrl</t>
   </si>
   <si>
     <t>- questionText must not be empty</t>
@@ -182,10 +194,10 @@
     <t>- For SHORT/LONG types, leave options empty and put the expected answer in correctAnswer</t>
   </si>
   <si>
-    <t>- marks must be a positive number</t>
-  </si>
-  <si>
     <t>- difficulty should be EASY, MEDIUM, or HARD</t>
+  </si>
+  <si>
+    <t>- imageUrl must be a direct, publicly accessible image link (e.g. ending in .png/.jpg) if provided</t>
   </si>
 </sst>
 </file>
@@ -587,19 +599,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="40" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="6" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -624,187 +636,211 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="E4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>14</v>
-      </c>
       <c r="H8" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -815,7 +851,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -824,12 +860,12 @@
   <sheetData>
     <row r="1" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -837,7 +873,7 @@
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -845,7 +881,7 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -853,7 +889,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -861,7 +897,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -869,7 +905,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -877,7 +913,7 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -885,7 +921,7 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -893,52 +929,60 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>